<commit_message>
chore: sync outstanding local changes (CLAUDE.md cleanup, catalog-sync tooling, settings)
Trims and reorganizes root/harkuhh CLAUDE.md for conciseness, adds .vercel and
__pycache__ to .gitignore, updates local Claude settings permissions, and adds
the weekly vendor catalog-sync tooling (diff.py + snapshots) that was sitting
uncommitted in harkuhh/scratchpad-sync/.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Affiliate_Overzicht.xlsx
+++ b/Affiliate_Overzicht.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affiliate Overzicht" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📖 Hoe te gebruiken" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Affiliate Overzicht'!$A$1:$J$12</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
 </file>
@@ -95,7 +97,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +114,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF0F4FF"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0F4FF"/>
+        <bgColor rgb="FFF0F4FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +157,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -216,6 +224,21 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -529,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="11" min="1" max="1"/>
@@ -575,7 +598,7 @@
           <t>🔗 Affiliate Link</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>📅 Geldig tot</t>
         </is>
@@ -627,7 +650,7 @@
           <t>https://engwe.com/?ref=uzjsbqmm</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>Geen einddatum</t>
         </is>
@@ -649,114 +672,404 @@
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1" s="12">
-      <c r="A3" s="17" t="n"/>
-      <c r="B3" s="17" t="n"/>
-      <c r="C3" s="17" t="n"/>
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Amazon Associates</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>E-bikes + accessoires (breed assortiment)</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Affiliate netwerk</t>
+        </is>
+      </c>
       <c r="D3" s="18" t="n"/>
       <c r="E3" s="18" t="n"/>
-      <c r="F3" s="17" t="n"/>
-      <c r="H3" s="18" t="n"/>
-      <c r="I3" s="18" t="n"/>
-      <c r="J3" s="17" t="n"/>
+      <c r="F3" s="23" t="n"/>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>n.v.t.</t>
+        </is>
+      </c>
+      <c r="H3" s="18" t="inlineStr">
+        <is>
+          <t>24 uur</t>
+        </is>
+      </c>
+      <c r="I3" s="18" t="inlineStr">
+        <is>
+          <t>Nog aanmelden</t>
+        </is>
+      </c>
+      <c r="J3" s="17" t="inlineStr">
+        <is>
+          <t>Aanmelden: affiliate-program.amazon.com. Lage commissie (~3%) maar hoge conversie en dekt merken zonder eigen programma.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="21.75" customHeight="1" s="12">
-      <c r="A4" s="14" t="n"/>
-      <c r="B4" s="14" t="n"/>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="15" t="n"/>
-      <c r="E4" s="15" t="n"/>
-      <c r="F4" s="14" t="n"/>
-      <c r="H4" s="15" t="n"/>
-      <c r="I4" s="15" t="n"/>
-      <c r="J4" s="14" t="n"/>
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>CJ Affiliate</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Toegang tot meerdere retailers/merken</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Affiliate netwerk</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="n"/>
+      <c r="E4" s="25" t="n"/>
+      <c r="F4" s="26" t="n"/>
+      <c r="G4" s="27" t="inlineStr">
+        <is>
+          <t>n.v.t.</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="inlineStr">
+        <is>
+          <t>Per merchant</t>
+        </is>
+      </c>
+      <c r="I4" s="25" t="inlineStr">
+        <is>
+          <t>Nog aanmelden</t>
+        </is>
+      </c>
+      <c r="J4" s="24" t="inlineStr">
+        <is>
+          <t>Aanmelden: cj.com/publishers. Groot netwerk, per merchant apart goedkeuring aanvragen.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="21.75" customHeight="1" s="12">
-      <c r="A5" s="17" t="n"/>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="17" t="n"/>
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Awin</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Toegang tot meerdere retailers/merken</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Affiliate netwerk</t>
+        </is>
+      </c>
       <c r="D5" s="18" t="n"/>
       <c r="E5" s="18" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="H5" s="18" t="n"/>
-      <c r="I5" s="18" t="n"/>
-      <c r="J5" s="17" t="n"/>
+      <c r="F5" s="23" t="n"/>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>n.v.t.</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Per merchant</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>Nog aanmelden</t>
+        </is>
+      </c>
+      <c r="J5" s="17" t="inlineStr">
+        <is>
+          <t>Aanmelden: awin.com. Let op: eenmalige aanmeldkosten die je terugkrijgt bij eerste uitbetaling.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="21.75" customHeight="1" s="12">
-      <c r="A6" s="14" t="n"/>
-      <c r="B6" s="14" t="n"/>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="15" t="n"/>
-      <c r="E6" s="15" t="n"/>
-      <c r="F6" s="14" t="n"/>
-      <c r="H6" s="15" t="n"/>
-      <c r="I6" s="15" t="n"/>
-      <c r="J6" s="14" t="n"/>
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>eBay Partner Network</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Nieuwe + refurbished e-bikes</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>Affiliate netwerk</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="n"/>
+      <c r="E6" s="25" t="n"/>
+      <c r="F6" s="26" t="n"/>
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>n.v.t.</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>24 uur</t>
+        </is>
+      </c>
+      <c r="I6" s="25" t="inlineStr">
+        <is>
+          <t>Nog aanmelden</t>
+        </is>
+      </c>
+      <c r="J6" s="24" t="inlineStr">
+        <is>
+          <t>Aanmelden: partnernetwork.ebay.com. Sterk voor refurbished en uitverkochte modellen (long-tail zoekverkeer).</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="21.75" customHeight="1" s="12">
-      <c r="A7" s="17" t="n"/>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="17" t="n"/>
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>REI</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>E-bikes van meerdere merken</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>Retailer (multi-merk)</t>
+        </is>
+      </c>
       <c r="D7" s="18" t="n"/>
       <c r="E7" s="18" t="n"/>
-      <c r="F7" s="17" t="n"/>
-      <c r="H7" s="18" t="n"/>
-      <c r="I7" s="18" t="n"/>
-      <c r="J7" s="17" t="n"/>
+      <c r="F7" s="23" t="n"/>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>n.v.t.</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>Nog checken</t>
+        </is>
+      </c>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>Nog aanmelden</t>
+        </is>
+      </c>
+      <c r="J7" s="17" t="inlineStr">
+        <is>
+          <t>Loopt via een affiliate netwerk (netwerk bevestigen bij aanmelding). Sterke merkautoriteit in de VS.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="21.75" customHeight="1" s="12">
-      <c r="A8" s="14" t="n"/>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="15" t="n"/>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="H8" s="15" t="n"/>
-      <c r="I8" s="15" t="n"/>
-      <c r="J8" s="14" t="n"/>
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Best Buy</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>E-bikes van meerdere merken</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>Retailer (multi-merk)</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="26" t="n"/>
+      <c r="G8" s="27" t="inlineStr">
+        <is>
+          <t>n.v.t.</t>
+        </is>
+      </c>
+      <c r="H8" s="25" t="inlineStr">
+        <is>
+          <t>Nog checken</t>
+        </is>
+      </c>
+      <c r="I8" s="25" t="inlineStr">
+        <is>
+          <t>Nog aanmelden</t>
+        </is>
+      </c>
+      <c r="J8" s="24" t="inlineStr">
+        <is>
+          <t>Loopt via een affiliate netwerk (netwerk bevestigen bij aanmelding). Breed assortiment mainstream merken.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="21.75" customHeight="1" s="12">
-      <c r="A9" s="17" t="n"/>
-      <c r="B9" s="17" t="n"/>
-      <c r="C9" s="17" t="n"/>
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Walmart</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>E-bikes van meerdere merken</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Retailer (multi-merk)</t>
+        </is>
+      </c>
       <c r="D9" s="18" t="n"/>
       <c r="E9" s="18" t="n"/>
-      <c r="F9" s="17" t="n"/>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="18" t="n"/>
-      <c r="J9" s="17" t="n"/>
+      <c r="F9" s="23" t="n"/>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>n.v.t.</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>Nog checken</t>
+        </is>
+      </c>
+      <c r="I9" s="18" t="inlineStr">
+        <is>
+          <t>Nog aanmelden</t>
+        </is>
+      </c>
+      <c r="J9" s="17" t="inlineStr">
+        <is>
+          <t>Loopt via een affiliate netwerk (netwerk bevestigen bij aanmelding). Dekt het budget-segment.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="21.75" customHeight="1" s="12">
-      <c r="A10" s="14" t="n"/>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="14" t="n"/>
-      <c r="H10" s="15" t="n"/>
-      <c r="I10" s="15" t="n"/>
-      <c r="J10" s="14" t="n"/>
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Backcountry</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>E-bikes en outdoor gear</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>Retailer (multi-merk)</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="n"/>
+      <c r="E10" s="25" t="n"/>
+      <c r="F10" s="26" t="n"/>
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>n.v.t.</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="inlineStr">
+        <is>
+          <t>Nog checken</t>
+        </is>
+      </c>
+      <c r="I10" s="25" t="inlineStr">
+        <is>
+          <t>Nog aanmelden</t>
+        </is>
+      </c>
+      <c r="J10" s="24" t="inlineStr">
+        <is>
+          <t>Loopt via een affiliate netwerk (netwerk bevestigen bij aanmelding). Meer premium/outdoor gericht.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="21.75" customHeight="1" s="12">
-      <c r="A11" s="17" t="n"/>
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="17" t="n"/>
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Skimlinks</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Automatische link-conversie (vangnet)</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Vangnet netwerk</t>
+        </is>
+      </c>
       <c r="D11" s="18" t="n"/>
       <c r="E11" s="18" t="n"/>
-      <c r="F11" s="17" t="n"/>
-      <c r="H11" s="18" t="n"/>
-      <c r="I11" s="18" t="n"/>
-      <c r="J11" s="17" t="n"/>
+      <c r="F11" s="23" t="n"/>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>n.v.t.</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>Per merchant</t>
+        </is>
+      </c>
+      <c r="I11" s="18" t="inlineStr">
+        <is>
+          <t>Nog aanmelden</t>
+        </is>
+      </c>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>Aanmelden: skimlinks.com. Zet links naar merchants zonder eigen deal alsnog om. Lagere marge, maar monetiseert de restcatalogus.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="21.75" customHeight="1" s="12">
-      <c r="A12" s="14" t="n"/>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="15" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="14" t="n"/>
-      <c r="H12" s="15" t="n"/>
-      <c r="I12" s="15" t="n"/>
-      <c r="J12" s="14" t="n"/>
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Sovrn Commerce</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Automatische link-conversie (vangnet)</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>Vangnet netwerk</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="n"/>
+      <c r="E12" s="25" t="n"/>
+      <c r="F12" s="26" t="n"/>
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>n.v.t.</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="inlineStr">
+        <is>
+          <t>Per merchant</t>
+        </is>
+      </c>
+      <c r="I12" s="25" t="inlineStr">
+        <is>
+          <t>Nog aanmelden</t>
+        </is>
+      </c>
+      <c r="J12" s="24" t="inlineStr">
+        <is>
+          <t>Aanmelden: sovrn.com/commerce. Alternatief voor Skimlinks, vergelijk de voorwaarden voordat je kiest.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="21.75" customHeight="1" s="12">
       <c r="A13" s="17" t="n"/>
@@ -868,7 +1181,128 @@
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="14" t="n"/>
     </row>
+    <row r="23" ht="21.75" customHeight="1" s="12">
+      <c r="A23" s="17" t="n"/>
+      <c r="B23" s="17" t="n"/>
+      <c r="C23" s="17" t="n"/>
+      <c r="D23" s="18" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="23" t="n"/>
+      <c r="G23" s="11" t="n"/>
+      <c r="H23" s="18" t="n"/>
+      <c r="I23" s="18" t="n"/>
+      <c r="J23" s="17" t="n"/>
+    </row>
+    <row r="24" ht="21.75" customHeight="1" s="12">
+      <c r="A24" s="24" t="n"/>
+      <c r="B24" s="24" t="n"/>
+      <c r="C24" s="24" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="25" t="n"/>
+      <c r="F24" s="26" t="n"/>
+      <c r="G24" s="27" t="n"/>
+      <c r="H24" s="25" t="n"/>
+      <c r="I24" s="25" t="n"/>
+      <c r="J24" s="24" t="n"/>
+    </row>
+    <row r="25" ht="21.75" customHeight="1" s="12">
+      <c r="A25" s="17" t="n"/>
+      <c r="B25" s="17" t="n"/>
+      <c r="C25" s="17" t="n"/>
+      <c r="D25" s="18" t="n"/>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="23" t="n"/>
+      <c r="G25" s="11" t="n"/>
+      <c r="H25" s="18" t="n"/>
+      <c r="I25" s="18" t="n"/>
+      <c r="J25" s="17" t="n"/>
+    </row>
+    <row r="26" ht="21.75" customHeight="1" s="12">
+      <c r="A26" s="24" t="n"/>
+      <c r="B26" s="24" t="n"/>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="25" t="n"/>
+      <c r="E26" s="25" t="n"/>
+      <c r="F26" s="26" t="n"/>
+      <c r="G26" s="27" t="n"/>
+      <c r="H26" s="25" t="n"/>
+      <c r="I26" s="25" t="n"/>
+      <c r="J26" s="24" t="n"/>
+    </row>
+    <row r="27" ht="21.75" customHeight="1" s="12">
+      <c r="A27" s="17" t="n"/>
+      <c r="B27" s="17" t="n"/>
+      <c r="C27" s="17" t="n"/>
+      <c r="D27" s="18" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="23" t="n"/>
+      <c r="G27" s="11" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="18" t="n"/>
+      <c r="J27" s="17" t="n"/>
+    </row>
+    <row r="28" ht="21.75" customHeight="1" s="12">
+      <c r="A28" s="24" t="n"/>
+      <c r="B28" s="24" t="n"/>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="25" t="n"/>
+      <c r="E28" s="25" t="n"/>
+      <c r="F28" s="26" t="n"/>
+      <c r="G28" s="27" t="n"/>
+      <c r="H28" s="25" t="n"/>
+      <c r="I28" s="25" t="n"/>
+      <c r="J28" s="24" t="n"/>
+    </row>
+    <row r="29" ht="21.75" customHeight="1" s="12">
+      <c r="A29" s="17" t="n"/>
+      <c r="B29" s="17" t="n"/>
+      <c r="C29" s="17" t="n"/>
+      <c r="D29" s="18" t="n"/>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="23" t="n"/>
+      <c r="G29" s="11" t="n"/>
+      <c r="H29" s="18" t="n"/>
+      <c r="I29" s="18" t="n"/>
+      <c r="J29" s="17" t="n"/>
+    </row>
+    <row r="30" ht="21.75" customHeight="1" s="12">
+      <c r="A30" s="24" t="n"/>
+      <c r="B30" s="24" t="n"/>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="25" t="n"/>
+      <c r="E30" s="25" t="n"/>
+      <c r="F30" s="26" t="n"/>
+      <c r="G30" s="27" t="n"/>
+      <c r="H30" s="25" t="n"/>
+      <c r="I30" s="25" t="n"/>
+      <c r="J30" s="24" t="n"/>
+    </row>
+    <row r="31" ht="21.75" customHeight="1" s="12">
+      <c r="A31" s="17" t="n"/>
+      <c r="B31" s="17" t="n"/>
+      <c r="C31" s="17" t="n"/>
+      <c r="D31" s="18" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="F31" s="23" t="n"/>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="18" t="n"/>
+      <c r="I31" s="18" t="n"/>
+      <c r="J31" s="17" t="n"/>
+    </row>
+    <row r="32" ht="21.75" customHeight="1" s="12">
+      <c r="A32" s="24" t="n"/>
+      <c r="B32" s="24" t="n"/>
+      <c r="C32" s="24" t="n"/>
+      <c r="D32" s="25" t="n"/>
+      <c r="E32" s="25" t="n"/>
+      <c r="F32" s="26" t="n"/>
+      <c r="G32" s="27" t="n"/>
+      <c r="H32" s="25" t="n"/>
+      <c r="I32" s="25" t="n"/>
+      <c r="J32" s="24" t="n"/>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:J12"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>